<commit_message>
Update admin dashboard and event features
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="184">
   <si>
     <t>id</t>
   </si>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t>100</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1540575467063-178a50c2df87?auto=format&amp;fit=crop&amp;w=900&amp;q=82&amp;utm_source=excel-event-hub&amp;utm_medium=referral</t>
   </si>
   <si>
     <t>[]</t>
@@ -1432,22 +1435,22 @@
         <v>109</v>
       </c>
       <c r="M8" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="N8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="O8" t="s">
         <v>38</v>
       </c>
       <c r="P8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="R8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="S8" t="s">
         <v>38</v>
@@ -1461,37 +1464,37 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J9" t="s">
         <v>74</v>
       </c>
       <c r="K9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L9" t="s">
         <v>97</v>
@@ -1500,13 +1503,13 @@
         <v>33</v>
       </c>
       <c r="N9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q9" t="s">
         <v>37</v>
@@ -1526,37 +1529,37 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J10" t="s">
         <v>48</v>
       </c>
       <c r="K10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="L10" t="s">
         <v>32</v>
@@ -1565,13 +1568,13 @@
         <v>33</v>
       </c>
       <c r="N10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q10" t="s">
         <v>37</v>
@@ -1591,52 +1594,52 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J11" t="s">
         <v>74</v>
       </c>
       <c r="K11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="M11" t="s">
         <v>33</v>
       </c>
       <c r="N11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Q11" t="s">
         <v>37</v>
@@ -1656,31 +1659,31 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C12" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H12" t="s">
         <v>72</v>
       </c>
       <c r="I12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J12" t="s">
         <v>87</v>
@@ -1689,19 +1692,19 @@
         <v>49</v>
       </c>
       <c r="L12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M12" t="s">
         <v>33</v>
       </c>
       <c r="N12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="Q12" t="s">
         <v>37</v>
@@ -1721,52 +1724,52 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K13" t="s">
         <v>31</v>
       </c>
       <c r="L13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M13" t="s">
         <v>33</v>
       </c>
       <c r="N13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O13" t="s">
         <v>35</v>
       </c>
       <c r="P13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q13" t="s">
         <v>37</v>
@@ -1786,52 +1789,52 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
       </c>
       <c r="K14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M14" t="s">
         <v>33</v>
       </c>
       <c r="N14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O14" t="s">
         <v>77</v>
       </c>
       <c r="P14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q14" t="s">
         <v>37</v>
@@ -1851,6 +1854,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>